<commit_message>
aligning exerzitien-kalatog in DE and EN
</commit_message>
<xml_diff>
--- a/translations_slugs_excel.xlsx
+++ b/translations_slugs_excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j.roe.AD\Documents\Code\online-exerzitien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{326490C4-484F-4DA6-BFCA-8B1473D456DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{A262E5F1-E1F2-4F0E-BF94-823AE7D7A721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2E021386-6AA5-49E3-9641-496B4BB9F9EB}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Tabelle1" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="ExterneDaten_1" localSheetId="0" hidden="1">translations_and_slugs_wide!$A$1:$Q$14</definedName>
+    <definedName name="ExterneDaten_1" localSheetId="0" hidden="1">translations_and_slugs_wide!$A$1:$Q$17</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="226">
   <si>
     <t>Column1</t>
   </si>
@@ -627,16 +627,126 @@
   </si>
   <si>
     <t>mua-vong</t>
+  </si>
+  <si>
+    <t>url</t>
+  </si>
+  <si>
+    <t>mailchimp (old)</t>
+  </si>
+  <si>
+    <t>https://retraites.carmes-paris.org/</t>
+  </si>
+  <si>
+    <t>http://www.exerzitien-online.karmel.at/</t>
+  </si>
+  <si>
+    <t>prefix</t>
+  </si>
+  <si>
+    <t>exerzitien-online</t>
+  </si>
+  <si>
+    <t>http://www.retiro-online.karmel.at/</t>
+  </si>
+  <si>
+    <t>retiro-online</t>
+  </si>
+  <si>
+    <t>http://www.esercizi-online.karmel.at/</t>
+  </si>
+  <si>
+    <t>esercizi-online</t>
+  </si>
+  <si>
+    <t>http://www.retreat-online.karmel.at/</t>
+  </si>
+  <si>
+    <t>retreat-online</t>
+  </si>
+  <si>
+    <t>http://www.rekolekcje-online.karmel.at/</t>
+  </si>
+  <si>
+    <t>rekolekcje-online</t>
+  </si>
+  <si>
+    <t>http://www.retraite-arabe.karmel.at/</t>
+  </si>
+  <si>
+    <t>retraite-arabe</t>
+  </si>
+  <si>
+    <t>http://webretiro.karmel.at/</t>
+  </si>
+  <si>
+    <t>webretiro</t>
+  </si>
+  <si>
+    <t>http://www.zaixian-tuixing.karmel.at/</t>
+  </si>
+  <si>
+    <t>zaixian-tuixing</t>
+  </si>
+  <si>
+    <t>http://exercicie-online.karmel.at/</t>
+  </si>
+  <si>
+    <t>exercicie-online</t>
+  </si>
+  <si>
+    <t>http://www.online-duhovne.karmel.at/</t>
+  </si>
+  <si>
+    <t>online-duhovne</t>
+  </si>
+  <si>
+    <t>http://www.online-lelkigyakorlat.karmel.at/</t>
+  </si>
+  <si>
+    <t>online-lelkigyakorlat</t>
+  </si>
+  <si>
+    <t>http://www.irtir-karmelitan-onlajn.karmel.at/</t>
+  </si>
+  <si>
+    <t>irtir-karmelitan-onlajn</t>
+  </si>
+  <si>
+    <t>http://www.retraitenl.karmel.at/</t>
+  </si>
+  <si>
+    <t>retraitenl</t>
+  </si>
+  <si>
+    <t>http://www.reculegere-online.karmel.at/</t>
+  </si>
+  <si>
+    <t>reculegere-online</t>
+  </si>
+  <si>
+    <t>http://www.tinh-tam-cat-minh.karmel.at/</t>
+  </si>
+  <si>
+    <t>tinh-tam-cat-minh</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -659,14 +769,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="17">
@@ -761,8 +874,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A2E9711A-6B18-4BE2-9119-6EA99673A870}" name="translations_and_slugs_wide" displayName="translations_and_slugs_wide" ref="A1:Q14" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:Q14" xr:uid="{A2E9711A-6B18-4BE2-9119-6EA99673A870}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A2E9711A-6B18-4BE2-9119-6EA99673A870}" name="translations_and_slugs_wide" displayName="translations_and_slugs_wide" ref="A1:Q17" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:Q17" xr:uid="{A2E9711A-6B18-4BE2-9119-6EA99673A870}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{C155324F-D559-4756-BC5A-54B2C4883BA6}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{1FB92865-EB92-470A-BB84-12C5C301FA71}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="15"/>
@@ -1103,7 +1216,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8674EE7-C218-49D1-AA6C-93D997160BE5}">
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
@@ -1867,10 +1980,146 @@
         <v>191</v>
       </c>
     </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="O15" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="Q15" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1"/>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="L17" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="M17" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="N17" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="O17" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="P17" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="Q17" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G15" r:id="rId1" xr:uid="{EEBBFA33-DE06-470A-8307-8E58FBE6F43C}"/>
+    <hyperlink ref="J15" r:id="rId2" xr:uid="{FD02D054-7139-4D5B-AAF4-3824B8023DF9}"/>
+    <hyperlink ref="K15" r:id="rId3" xr:uid="{D0FFAABA-4106-491B-AEE4-DE271D6F622D}"/>
+    <hyperlink ref="L15" r:id="rId4" xr:uid="{600A81CC-1118-4BE8-823E-1CF7E2806409}"/>
+    <hyperlink ref="M15" r:id="rId5" xr:uid="{9AAF5863-4CC5-4D2A-9F47-F8AB4881F86B}"/>
+    <hyperlink ref="N15" r:id="rId6" xr:uid="{F2BBA5C5-55C7-466F-87A5-E9A91AE1CF79}"/>
+    <hyperlink ref="O15" r:id="rId7" xr:uid="{4B3A7FDC-39AB-4069-93AD-F7910F0A2AB8}"/>
+    <hyperlink ref="P15" r:id="rId8" xr:uid="{23A299A0-E4E1-4951-AF72-C57F0537B27C}"/>
+    <hyperlink ref="Q15" r:id="rId9" xr:uid="{D5756BE7-B955-453A-A286-DCB0438717BF}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId10"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
switch exerzitien_katalog with retreat_overview
</commit_message>
<xml_diff>
--- a/translations_slugs_excel.xlsx
+++ b/translations_slugs_excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j.roe.AD\Documents\Code\online-exerzitien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{A262E5F1-E1F2-4F0E-BF94-823AE7D7A721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{3808BAAB-1B95-4C7B-9EA1-762C58D7BAF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2E021386-6AA5-49E3-9641-496B4BB9F9EB}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="228">
   <si>
     <t>Column1</t>
   </si>
@@ -729,6 +729,12 @@
   </si>
   <si>
     <t>tinh-tam-cat-minh</t>
+  </si>
+  <si>
+    <t>Došašće</t>
+  </si>
+  <si>
+    <t>dosasce</t>
   </si>
 </sst>
 </file>
@@ -1591,7 +1597,7 @@
         <v>95</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>95</v>
+        <v>226</v>
       </c>
       <c r="M7" s="1" t="s">
         <v>95</v>
@@ -1962,7 +1968,7 @@
         <v>93</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>93</v>
+        <v>227</v>
       </c>
       <c r="M14" s="1" t="s">
         <v>93</v>
@@ -2118,8 +2124,9 @@
     <hyperlink ref="Q15" r:id="rId9" xr:uid="{D5756BE7-B955-453A-A286-DCB0438717BF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId10"/>
   <tableParts count="1">
-    <tablePart r:id="rId10"/>
+    <tablePart r:id="rId11"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
hu & mt initial
</commit_message>
<xml_diff>
--- a/translations_slugs_excel.xlsx
+++ b/translations_slugs_excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j.roe.AD\Documents\Code\online-exerzitien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F934A069-AC63-48E7-A2DF-C45F4EF3A1A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65180396-A72D-4C48-B285-B9B154208278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="230">
   <si>
     <t>Column1</t>
   </si>
@@ -724,6 +724,9 @@
   </si>
   <si>
     <t>https://karmel.us6.list-manage.com/subscribe?u=7c9d2aa0ecc1fde64fd44bc67&amp;id=3eb40fe31e</t>
+  </si>
+  <si>
+    <t>https://karmel.us6.list-manage.com/subscribe?u=7c9d2aa0ecc1fde64fd44bc67&amp;id=33079f5616</t>
   </si>
 </sst>
 </file>
@@ -1897,6 +1900,9 @@
       <c r="L16" t="s">
         <v>228</v>
       </c>
+      <c r="N16" t="s">
+        <v>229</v>
+      </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">

</xml_diff>